<commit_message>
Calculadora: selección de países, IIBB Argentina, plan RM (SaaS/EBOX), volumen por pacientes y explicaciones
Aplicado en presentacion.html y en modelo.xlsx (hoja Calculadora).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modelo.xlsx
+++ b/modelo.xlsx
@@ -166,7 +166,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -213,6 +213,12 @@
     <xf numFmtId="3" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -235,10 +241,10 @@
     <xf numFmtId="3" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -362,6 +368,11 @@
         <t>Costo fijo que Rumotech traslada a NexoLibre por modalidad activa. Es en USD y NO varía por país: por eso fija un precio mínimo viable por estudio en cada mercado.</t>
       </text>
     </comment>
+    <comment ref="G10" authorId="0" shapeId="0">
+      <text>
+        <t>Ingresos Brutos: impuesto provincial argentino sobre el ingreso bruto (~3% según provincia/actividad). Reduce el margen. En los demás países es 0. VALIDAR con contador local.</t>
+      </text>
+    </comment>
     <comment ref="D11" authorId="0" shapeId="0">
       <text>
         <t>Valor de referencia de un estudio de RM en USD (estimado, orientativo). Argentina/Colombia usan el reembolso realizado en USD (bajo/volátil), no el precio particular. VALIDAR con aranceles locales reales.</t>
@@ -375,6 +386,126 @@
     <comment ref="B23" authorId="0" shapeId="0">
       <text>
         <t>Mínimo mensual por modalidad. Clave en mercados baratos (Argentina/Colombia): garantiza cubrir el costo fijo de Rumotech aunque el volumen sea bajo. Puede calibrarse por país.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Modelo</author>
+  </authors>
+  <commentList>
+    <comment ref="B5" authorId="0" shapeId="0">
+      <text>
+        <t>País a simular. Toma precio, IVA, IIBB y renta desde la hoja Supuestos.</t>
+      </text>
+    </comment>
+    <comment ref="B6" authorId="0" shapeId="0">
+      <text>
+        <t>Ubicaciones físicas del cliente. El costo por modalidad se cobra en cada sede.</t>
+      </text>
+    </comment>
+    <comment ref="B7" authorId="0" shapeId="0">
+      <text>
+        <t>SaaS Full + Cryogenics: RM cuesta el fijo por sede. EBOX Full: RM cuesta por resonador (celda de abajo).</t>
+      </text>
+    </comment>
+    <comment ref="B8" authorId="0" shapeId="0">
+      <text>
+        <t>Costo que Rumotech cobra por cada resonador con EBOX Full. Solo aplica si el plan RM = EBOX Full.</t>
+      </text>
+    </comment>
+    <comment ref="B9" authorId="0" shapeId="0">
+      <text>
+        <t>Por equipos: volumen = equipos × estudios/equipo. Por pacientes: volumen = pacientes × coeficiente (como calculan los centros).</t>
+      </text>
+    </comment>
+    <comment ref="B10" authorId="0" shapeId="0">
+      <text>
+        <t>Solo se usa si el método = Por pacientes.</t>
+      </text>
+    </comment>
+    <comment ref="B11" authorId="0" shapeId="0">
+      <text>
+        <t>Prestaciones promedio por paciente. Prestaciones/sede = pacientes × coeficiente.</t>
+      </text>
+    </comment>
+    <comment ref="E14" authorId="0" shapeId="0">
+      <text>
+        <t>RM: con SaaS+Cryo = costo fijo por sede; con EBOX = (costo anual EBOX ÷ 12) × resonadores de la sede.</t>
+      </text>
+    </comment>
+    <comment ref="A22" authorId="0" shapeId="0">
+      <text>
+        <t>Modalidades distintas por sede. Cada una paga el costo fijo (salvo RM con EBOX).</t>
+      </text>
+    </comment>
+    <comment ref="A23" authorId="0" shapeId="0">
+      <text>
+        <t>Por equipos = Σ equipos × estudios. Por pacientes = pacientes × coeficiente.</t>
+      </text>
+    </comment>
+    <comment ref="A24" authorId="0" shapeId="0">
+      <text>
+        <t>Prestaciones por sede × número de sedes.</t>
+      </text>
+    </comment>
+    <comment ref="A25" authorId="0" shapeId="0">
+      <text>
+        <t>Suma de costos por modalidad y sede. RM con EBOX = (costo anual÷12) × resonadores.</t>
+      </text>
+    </comment>
+    <comment ref="A26" authorId="0" shapeId="0">
+      <text>
+        <t>Costo total ÷ prestaciones. Baja con la densidad de equipos/sedes.</t>
+      </text>
+    </comment>
+    <comment ref="A27" authorId="0" shapeId="0">
+      <text>
+        <t>Precio de venta al centro, sin IVA. Se toma de Supuestos según el país.</t>
+      </text>
+    </comment>
+    <comment ref="A28" authorId="0" shapeId="0">
+      <text>
+        <t>Precio × (1 + IVA). El IVA es pass-through: neutro para la renta.</t>
+      </text>
+    </comment>
+    <comment ref="A29" authorId="0" shapeId="0">
+      <text>
+        <t>Volumen total × precio neto de IVA.</t>
+      </text>
+    </comment>
+    <comment ref="A30" authorId="0" shapeId="0">
+      <text>
+        <t>Impuesto provincial argentino sobre el ingreso bruto. Reduce el margen. 0 en los demás países.</t>
+      </text>
+    </comment>
+    <comment ref="A31" authorId="0" shapeId="0">
+      <text>
+        <t>Ingreso − costo Rumotech − IIBB.</t>
+      </text>
+    </comment>
+    <comment ref="A32" authorId="0" shapeId="0">
+      <text>
+        <t>Alícuota del país sobre el margen operativo positivo.</t>
+      </text>
+    </comment>
+    <comment ref="A33" authorId="0" shapeId="0">
+      <text>
+        <t>Costo único por resonador: SaaS+Cryo 150, EBOX 500. No es recurrente; no entra en la renta anual.</t>
+      </text>
+    </comment>
+    <comment ref="A34" authorId="0" shapeId="0">
+      <text>
+        <t>Margen operativo menos impuesto a la renta.</t>
+      </text>
+    </comment>
+    <comment ref="A35" authorId="0" shapeId="0">
+      <text>
+        <t>Renta pasiva anual que retiene NexoLibre.</t>
       </text>
     </comment>
   </commentList>
@@ -852,7 +983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -861,6 +992,7 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -953,6 +1085,12 @@
 (% del estudio)</t>
         </is>
       </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>IIBB %
+(Arg.)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
@@ -976,6 +1114,9 @@
         <f>IF(D11=0,0,E11/D11)</f>
         <v/>
       </c>
+      <c r="G11" s="14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
@@ -999,6 +1140,9 @@
         <f>IF(D12=0,0,E12/D12)</f>
         <v/>
       </c>
+      <c r="G12" s="14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
@@ -1022,6 +1166,9 @@
         <f>IF(D13=0,0,E13/D13)</f>
         <v/>
       </c>
+      <c r="G13" s="14" t="n">
+        <v>0.03</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="13" t="inlineStr">
@@ -1045,6 +1192,9 @@
         <f>IF(D14=0,0,E14/D14)</f>
         <v/>
       </c>
+      <c r="G14" s="14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
@@ -1067,6 +1217,9 @@
       <c r="F15" s="17">
         <f>IF(D15=0,0,E15/D15)</f>
         <v/>
+      </c>
+      <c r="G15" s="14" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -1140,11 +1293,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
@@ -1154,14 +1307,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Calculadora de Escenarios — Sedes, Equipos y Rentabilidad por Cliente</t>
+          <t>Calculadora de Escenarios — Rentabilidad por Cliente</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Clave: el costo de Rumotech es USD 100 por MODALIDAD por SEDE — no por cantidad de equipos. Varios RM/CT en una sede diluyen el costo. Editá las celdas AZULES.</t>
+          <t>El costo de Rumotech es por MODALIDAD y por SEDE (no por equipo), salvo RM con EBOX (por resonador). Editá las celdas AZULES. Los comentarios (triángulo rojo) explican cada valor.</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1328,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>País</t>
+          <t>País (elegí de la lista)</t>
         </is>
       </c>
       <c r="B5" s="20" t="inlineStr">
@@ -1194,264 +1347,258 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Plan para RM</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>SaaS Full + Cryogenics</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>EBOX Full — costo anual por resonador (USD)</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Método de volumen</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>Por equipos</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Pacientes / mes por sede</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="n">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Coeficiente de exámenes por paciente</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Modalidad</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Equipos
 por sede</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>Estudios /
 equipo / mes</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>Modalidad
 activa</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E13" s="12" t="inlineStr">
         <is>
           <t>Costo Rumotech
 / sede (USD)</t>
         </is>
       </c>
-      <c r="F8" s="12" t="inlineStr">
+      <c r="F13" s="12" t="inlineStr">
         <is>
           <t>Volumen / sede
-(est./mes)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+(equipos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>Resonancia (RM)</t>
         </is>
       </c>
-      <c r="B9" s="21" t="n">
+      <c r="B14" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="21" t="n">
+      <c r="C14" s="21" t="n">
         <v>500</v>
       </c>
-      <c r="D9" s="22">
-        <f>IF(B9&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="E9" s="23">
-        <f>D9*Supuestos!$B$5</f>
-        <v/>
-      </c>
-      <c r="F9" s="24">
-        <f>B9*C9</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="D14" s="24">
+        <f>IF(B14&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="E14" s="25">
+        <f>IF(B14&gt;0,IF($B$7="EBOX Full",($B$8/12)*B14,Supuestos!$B$5),0)</f>
+        <v/>
+      </c>
+      <c r="F14" s="26">
+        <f>B14*C14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>Tomografía (CT)</t>
         </is>
       </c>
-      <c r="B10" s="21" t="n">
+      <c r="B15" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="21" t="n">
+      <c r="C15" s="21" t="n">
         <v>700</v>
       </c>
-      <c r="D10" s="22">
-        <f>IF(B10&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="E10" s="23">
-        <f>D10*Supuestos!$B$5</f>
-        <v/>
-      </c>
-      <c r="F10" s="24">
-        <f>B10*C10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="D15" s="24">
+        <f>IF(B15&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="E15" s="25">
+        <f>IF(B15&gt;0,Supuestos!$B$5,0)</f>
+        <v/>
+      </c>
+      <c r="F15" s="26">
+        <f>B15*C15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>Ultrasonido (US)</t>
         </is>
       </c>
-      <c r="B11" s="21" t="n">
+      <c r="B16" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="21" t="n">
+      <c r="C16" s="21" t="n">
         <v>1000</v>
       </c>
-      <c r="D11" s="22">
-        <f>IF(B11&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="E11" s="23">
-        <f>D11*Supuestos!$B$5</f>
-        <v/>
-      </c>
-      <c r="F11" s="24">
-        <f>B11*C11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="D16" s="24">
+        <f>IF(B16&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="E16" s="25">
+        <f>IF(B16&gt;0,Supuestos!$B$5,0)</f>
+        <v/>
+      </c>
+      <c r="F16" s="26">
+        <f>B16*C16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>Rayos X (RX)</t>
         </is>
       </c>
-      <c r="B12" s="21" t="n">
+      <c r="B17" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="C12" s="21" t="n">
+      <c r="C17" s="21" t="n">
         <v>1200</v>
       </c>
-      <c r="D12" s="22">
-        <f>IF(B12&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="E12" s="23">
-        <f>D12*Supuestos!$B$5</f>
-        <v/>
-      </c>
-      <c r="F12" s="24">
-        <f>B12*C12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="D17" s="24">
+        <f>IF(B17&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="E17" s="25">
+        <f>IF(B17&gt;0,Supuestos!$B$5,0)</f>
+        <v/>
+      </c>
+      <c r="F17" s="26">
+        <f>B17*C17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>Mamografía (MG)</t>
         </is>
       </c>
-      <c r="B13" s="21" t="n">
+      <c r="B18" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="C13" s="21" t="n">
+      <c r="C18" s="21" t="n">
         <v>300</v>
       </c>
-      <c r="D13" s="22">
-        <f>IF(B13&gt;0,1,0)</f>
-        <v/>
-      </c>
-      <c r="E13" s="23">
-        <f>D13*Supuestos!$B$5</f>
-        <v/>
-      </c>
-      <c r="F13" s="24">
-        <f>B13*C13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="25" t="inlineStr">
+      <c r="D18" s="24">
+        <f>IF(B18&gt;0,1,0)</f>
+        <v/>
+      </c>
+      <c r="E18" s="25">
+        <f>IF(B18&gt;0,Supuestos!$B$5,0)</f>
+        <v/>
+      </c>
+      <c r="F18" s="26">
+        <f>B18*C18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="27" t="inlineStr">
         <is>
           <t>Total por sede</t>
         </is>
       </c>
-      <c r="B14" s="26" t="n"/>
-      <c r="C14" s="26" t="n"/>
-      <c r="D14" s="27">
-        <f>SUM(D9:D13)</f>
-        <v/>
-      </c>
-      <c r="E14" s="28">
-        <f>SUM(E9:E13)</f>
-        <v/>
-      </c>
-      <c r="F14" s="29">
-        <f>SUM(F9:F13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="B19" s="28" t="n"/>
+      <c r="C19" s="28" t="n"/>
+      <c r="D19" s="29">
+        <f>SUM(D14:D18)</f>
+        <v/>
+      </c>
+      <c r="E19" s="30">
+        <f>SUM(E14:E18)</f>
+        <v/>
+      </c>
+      <c r="F19" s="31">
+        <f>SUM(F14:F18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>RESULTADOS DEL CLIENTE (todas las sedes)</t>
         </is>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Modalidades activas por sede</t>
-        </is>
-      </c>
-      <c r="E17" s="24">
-        <f>D14</f>
-        <v/>
-      </c>
-      <c r="F17" s="7" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Costo Rumotech mensual — total cliente (USD)</t>
-        </is>
-      </c>
-      <c r="E18" s="23">
-        <f>E14*B6</f>
-        <v/>
-      </c>
-      <c r="F18" s="7" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Volumen total de estudios / mes</t>
-        </is>
-      </c>
-      <c r="E19" s="24">
-        <f>F14*B6</f>
-        <v/>
-      </c>
-      <c r="F19" s="7" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Precio por estudio — país (USD)</t>
-        </is>
-      </c>
-      <c r="E20" s="30">
-        <f>INDEX(Supuestos!$E$11:$E$15,MATCH(B5,Supuestos!$A$11:$A$15,0))</f>
-        <v/>
-      </c>
-      <c r="F20" s="7" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Costo Rumotech EFECTIVO por estudio (USD)</t>
-        </is>
-      </c>
-      <c r="E21" s="31">
-        <f>IF((F14*B6)=0,0,(E14*B6)/(F14*B6))</f>
-        <v/>
-      </c>
-      <c r="F21" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Ingreso mensual — total cliente (USD)</t>
-        </is>
-      </c>
-      <c r="E22" s="23">
-        <f>F14*B6*INDEX(Supuestos!$E$11:$E$15,MATCH(B5,Supuestos!$A$11:$A$15,0))</f>
+          <t>Modalidades activas por sede</t>
+        </is>
+      </c>
+      <c r="E22" s="26">
+        <f>D19</f>
         <v/>
       </c>
       <c r="F22" s="7" t="n"/>
@@ -1459,11 +1606,11 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Margen bruto mensual (USD)</t>
-        </is>
-      </c>
-      <c r="E23" s="23">
-        <f>F14*B6*INDEX(Supuestos!$E$11:$E$15,MATCH(B5,Supuestos!$A$11:$A$15,0))-E14*B6</f>
+          <t>Prestaciones (estudios) por sede</t>
+        </is>
+      </c>
+      <c r="E23" s="26">
+        <f>IF($B$9="Por pacientes",$B$10*$B$11,F19)</f>
         <v/>
       </c>
       <c r="F23" s="7" t="n"/>
@@ -1471,11 +1618,11 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Imp. a la renta — país</t>
-        </is>
-      </c>
-      <c r="E24" s="32">
-        <f>INDEX(Supuestos!$C$11:$C$15,MATCH(B5,Supuestos!$A$11:$A$15,0))</f>
+          <t>Volumen total de prestaciones / mes</t>
+        </is>
+      </c>
+      <c r="E24" s="26">
+        <f>(IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6</f>
         <v/>
       </c>
       <c r="F24" s="7" t="n"/>
@@ -1483,11 +1630,11 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Renta neta mensual (USD)</t>
-        </is>
-      </c>
-      <c r="E25" s="23">
-        <f>(F14*B6*INDEX(Supuestos!$E$11:$E$15,MATCH(B5,Supuestos!$A$11:$A$15,0))-E14*B6)*(1-INDEX(Supuestos!$C$11:$C$15,MATCH(B5,Supuestos!$A$11:$A$15,0)))</f>
+          <t>Costo Rumotech mensual — total (USD)</t>
+        </is>
+      </c>
+      <c r="E25" s="25">
+        <f>E19*$B$6</f>
         <v/>
       </c>
       <c r="F25" s="7" t="n"/>
@@ -1495,54 +1642,177 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
+          <t>Costo Rumotech EFECTIVO por prestación (USD)</t>
+        </is>
+      </c>
+      <c r="E26" s="32">
+        <f>IF(((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)=0,0,(E19*$B$6)/((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6))</f>
+        <v/>
+      </c>
+      <c r="F26" s="7" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Precio por prestación — neto de IVA (USD)</t>
+        </is>
+      </c>
+      <c r="E27" s="33">
+        <f>INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))</f>
+        <v/>
+      </c>
+      <c r="F27" s="7" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Precio final al cliente c/ IVA (USD)</t>
+        </is>
+      </c>
+      <c r="E28" s="33">
+        <f>INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))*(1+INDEX(Supuestos!$B$11:$B$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))</f>
+        <v/>
+      </c>
+      <c r="F28" s="7" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Ingreso mensual — total (USD)</t>
+        </is>
+      </c>
+      <c r="E29" s="25">
+        <f>((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))</f>
+        <v/>
+      </c>
+      <c r="F29" s="7" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Ingresos Brutos (IIBB) mensual (USD)</t>
+        </is>
+      </c>
+      <c r="E30" s="25">
+        <f>(((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))</f>
+        <v/>
+      </c>
+      <c r="F30" s="7" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Margen operativo mensual (USD)</t>
+        </is>
+      </c>
+      <c r="E31" s="25">
+        <f>(((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))-(E19*$B$6)-((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))</f>
+        <v/>
+      </c>
+      <c r="F31" s="7" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Impuesto a la renta mensual (USD)</t>
+        </is>
+      </c>
+      <c r="E32" s="25">
+        <f>IF(((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))-(E19*$B$6)-((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))))&gt;0,((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))-(E19*$B$6)-((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))))*INDEX(Supuestos!$C$11:$C$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)),0)</f>
+        <v/>
+      </c>
+      <c r="F32" s="7" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Hardware (pago ÚNICO, USD)</t>
+        </is>
+      </c>
+      <c r="E33" s="25">
+        <f>IF($B$7="EBOX Full",500,150)*B14*$B$6</f>
+        <v/>
+      </c>
+      <c r="F33" s="7" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Renta neta mensual (USD)</t>
+        </is>
+      </c>
+      <c r="E34" s="25">
+        <f>((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))-(E19*$B$6)-((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))))-IF(((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))-(E19*$B$6)-((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))))&gt;0,((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))-(E19*$B$6)-((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))))*INDEX(Supuestos!$C$11:$C$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)),0)</f>
+        <v/>
+      </c>
+      <c r="F34" s="7" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
           <t>RENTA NETA ANUAL — total cliente (USD)</t>
         </is>
       </c>
-      <c r="E26" s="6">
-        <f>((F14*B6*INDEX(Supuestos!$E$11:$E$15,MATCH(B5,Supuestos!$A$11:$A$15,0))-E14*B6)*(1-INDEX(Supuestos!$C$11:$C$15,MATCH(B5,Supuestos!$A$11:$A$15,0))))*12</f>
-        <v/>
-      </c>
-      <c r="F26" s="7" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>El 'costo efectivo por estudio' cae al agregar equipos/sedes: ahí se ve cómo un cliente denso compensa un precio bajo (ej. Argentina).</t>
+      <c r="E35" s="6">
+        <f>(((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))-(E19*$B$6)-((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))))-IF(((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))-(E19*$B$6)-((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))))&gt;0,((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))-(E19*$B$6)-((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))))*INDEX(Supuestos!$C$11:$C$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)),0))*12</f>
+        <v/>
+      </c>
+      <c r="F35" s="7" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Ejercicios: cambiá el plan de RM (SaaS+Cryo vs EBOX), el método de volumen (equipos vs pacientes) o el país, y observá la renta.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="23">
-    <mergeCell ref="A17:D17"/>
+  <mergeCells count="31">
     <mergeCell ref="A23:D23"/>
     <mergeCell ref="A22:D22"/>
     <mergeCell ref="E24:F24"/>
-    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A29:D29"/>
     <mergeCell ref="E23:F23"/>
-    <mergeCell ref="A19:D19"/>
-    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="A28:D28"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="E28:F28"/>
     <mergeCell ref="A24:D24"/>
-    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="E27:F27"/>
     <mergeCell ref="A25:D25"/>
     <mergeCell ref="E26:F26"/>
-    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="E32:F32"/>
     <mergeCell ref="E25:F25"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A21:D21"/>
     <mergeCell ref="E22:F22"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A32:D32"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="3">
     <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Chile,Uruguay,Argentina,Colombia,USA"</formula1>
     </dataValidation>
+    <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"SaaS Full + Cryogenics,EBOX Full"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Por equipos,Por pacientes"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1658,87 +1928,87 @@
           <t>Bajo</t>
         </is>
       </c>
-      <c r="C5" s="24">
+      <c r="C5" s="26">
         <f>Supuestos!$B$18</f>
         <v/>
       </c>
-      <c r="D5" s="30">
+      <c r="D5" s="33">
         <f>Supuestos!$B$5/C5</f>
         <v/>
       </c>
-      <c r="E5" s="30">
+      <c r="E5" s="33">
         <f>Supuestos!$E$11</f>
         <v/>
       </c>
-      <c r="F5" s="30">
+      <c r="F5" s="33">
         <f>E5-D5</f>
         <v/>
       </c>
-      <c r="G5" s="32">
+      <c r="G5" s="34">
         <f>IF(E5=0,0,F5/E5)</f>
         <v/>
       </c>
-      <c r="H5" s="32">
+      <c r="H5" s="34">
         <f>Supuestos!$C$11</f>
         <v/>
       </c>
-      <c r="I5" s="30">
+      <c r="I5" s="33">
         <f>F5*(1-H5)</f>
         <v/>
       </c>
-      <c r="J5" s="23">
+      <c r="J5" s="25">
         <f>I5*C5</f>
         <v/>
       </c>
-      <c r="K5" s="23">
+      <c r="K5" s="25">
         <f>J5*12</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="33" t="inlineStr">
+      <c r="A6" s="35" t="inlineStr">
         <is>
           <t>Chile</t>
         </is>
       </c>
-      <c r="B6" s="33" t="inlineStr">
+      <c r="B6" s="35" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="C6" s="34">
+      <c r="C6" s="36">
         <f>Supuestos!$B$19</f>
         <v/>
       </c>
-      <c r="D6" s="35">
+      <c r="D6" s="37">
         <f>Supuestos!$B$5/C6</f>
         <v/>
       </c>
-      <c r="E6" s="35">
+      <c r="E6" s="37">
         <f>Supuestos!$E$11</f>
         <v/>
       </c>
-      <c r="F6" s="35">
+      <c r="F6" s="37">
         <f>E6-D6</f>
         <v/>
       </c>
-      <c r="G6" s="36">
+      <c r="G6" s="38">
         <f>IF(E6=0,0,F6/E6)</f>
         <v/>
       </c>
-      <c r="H6" s="36">
+      <c r="H6" s="38">
         <f>Supuestos!$C$11</f>
         <v/>
       </c>
-      <c r="I6" s="35">
+      <c r="I6" s="37">
         <f>F6*(1-H6)</f>
         <v/>
       </c>
-      <c r="J6" s="37">
+      <c r="J6" s="39">
         <f>I6*C6</f>
         <v/>
       </c>
-      <c r="K6" s="37">
+      <c r="K6" s="39">
         <f>J6*12</f>
         <v/>
       </c>
@@ -1754,39 +2024,39 @@
           <t>Alto</t>
         </is>
       </c>
-      <c r="C7" s="24">
+      <c r="C7" s="26">
         <f>Supuestos!$B$20</f>
         <v/>
       </c>
-      <c r="D7" s="30">
+      <c r="D7" s="33">
         <f>Supuestos!$B$5/C7</f>
         <v/>
       </c>
-      <c r="E7" s="30">
+      <c r="E7" s="33">
         <f>Supuestos!$E$11</f>
         <v/>
       </c>
-      <c r="F7" s="30">
+      <c r="F7" s="33">
         <f>E7-D7</f>
         <v/>
       </c>
-      <c r="G7" s="32">
+      <c r="G7" s="34">
         <f>IF(E7=0,0,F7/E7)</f>
         <v/>
       </c>
-      <c r="H7" s="32">
+      <c r="H7" s="34">
         <f>Supuestos!$C$11</f>
         <v/>
       </c>
-      <c r="I7" s="30">
+      <c r="I7" s="33">
         <f>F7*(1-H7)</f>
         <v/>
       </c>
-      <c r="J7" s="23">
+      <c r="J7" s="25">
         <f>I7*C7</f>
         <v/>
       </c>
-      <c r="K7" s="23">
+      <c r="K7" s="25">
         <f>J7*12</f>
         <v/>
       </c>
@@ -1802,87 +2072,87 @@
           <t>Bajo</t>
         </is>
       </c>
-      <c r="C8" s="24">
+      <c r="C8" s="26">
         <f>Supuestos!$B$18</f>
         <v/>
       </c>
-      <c r="D8" s="30">
+      <c r="D8" s="33">
         <f>Supuestos!$B$5/C8</f>
         <v/>
       </c>
-      <c r="E8" s="30">
+      <c r="E8" s="33">
         <f>Supuestos!$E$12</f>
         <v/>
       </c>
-      <c r="F8" s="30">
+      <c r="F8" s="33">
         <f>E8-D8</f>
         <v/>
       </c>
-      <c r="G8" s="32">
+      <c r="G8" s="34">
         <f>IF(E8=0,0,F8/E8)</f>
         <v/>
       </c>
-      <c r="H8" s="32">
+      <c r="H8" s="34">
         <f>Supuestos!$C$12</f>
         <v/>
       </c>
-      <c r="I8" s="30">
+      <c r="I8" s="33">
         <f>F8*(1-H8)</f>
         <v/>
       </c>
-      <c r="J8" s="23">
+      <c r="J8" s="25">
         <f>I8*C8</f>
         <v/>
       </c>
-      <c r="K8" s="23">
+      <c r="K8" s="25">
         <f>J8*12</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="33" t="inlineStr">
+      <c r="A9" s="35" t="inlineStr">
         <is>
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="B9" s="33" t="inlineStr">
+      <c r="B9" s="35" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="C9" s="34">
+      <c r="C9" s="36">
         <f>Supuestos!$B$19</f>
         <v/>
       </c>
-      <c r="D9" s="35">
+      <c r="D9" s="37">
         <f>Supuestos!$B$5/C9</f>
         <v/>
       </c>
-      <c r="E9" s="35">
+      <c r="E9" s="37">
         <f>Supuestos!$E$12</f>
         <v/>
       </c>
-      <c r="F9" s="35">
+      <c r="F9" s="37">
         <f>E9-D9</f>
         <v/>
       </c>
-      <c r="G9" s="36">
+      <c r="G9" s="38">
         <f>IF(E9=0,0,F9/E9)</f>
         <v/>
       </c>
-      <c r="H9" s="36">
+      <c r="H9" s="38">
         <f>Supuestos!$C$12</f>
         <v/>
       </c>
-      <c r="I9" s="35">
+      <c r="I9" s="37">
         <f>F9*(1-H9)</f>
         <v/>
       </c>
-      <c r="J9" s="37">
+      <c r="J9" s="39">
         <f>I9*C9</f>
         <v/>
       </c>
-      <c r="K9" s="37">
+      <c r="K9" s="39">
         <f>J9*12</f>
         <v/>
       </c>
@@ -1898,39 +2168,39 @@
           <t>Alto</t>
         </is>
       </c>
-      <c r="C10" s="24">
+      <c r="C10" s="26">
         <f>Supuestos!$B$20</f>
         <v/>
       </c>
-      <c r="D10" s="30">
+      <c r="D10" s="33">
         <f>Supuestos!$B$5/C10</f>
         <v/>
       </c>
-      <c r="E10" s="30">
+      <c r="E10" s="33">
         <f>Supuestos!$E$12</f>
         <v/>
       </c>
-      <c r="F10" s="30">
+      <c r="F10" s="33">
         <f>E10-D10</f>
         <v/>
       </c>
-      <c r="G10" s="32">
+      <c r="G10" s="34">
         <f>IF(E10=0,0,F10/E10)</f>
         <v/>
       </c>
-      <c r="H10" s="32">
+      <c r="H10" s="34">
         <f>Supuestos!$C$12</f>
         <v/>
       </c>
-      <c r="I10" s="30">
+      <c r="I10" s="33">
         <f>F10*(1-H10)</f>
         <v/>
       </c>
-      <c r="J10" s="23">
+      <c r="J10" s="25">
         <f>I10*C10</f>
         <v/>
       </c>
-      <c r="K10" s="23">
+      <c r="K10" s="25">
         <f>J10*12</f>
         <v/>
       </c>
@@ -1946,87 +2216,87 @@
           <t>Bajo</t>
         </is>
       </c>
-      <c r="C11" s="24">
+      <c r="C11" s="26">
         <f>Supuestos!$B$18</f>
         <v/>
       </c>
-      <c r="D11" s="30">
+      <c r="D11" s="33">
         <f>Supuestos!$B$5/C11</f>
         <v/>
       </c>
-      <c r="E11" s="30">
+      <c r="E11" s="33">
         <f>Supuestos!$E$13</f>
         <v/>
       </c>
-      <c r="F11" s="30">
+      <c r="F11" s="33">
         <f>E11-D11</f>
         <v/>
       </c>
-      <c r="G11" s="32">
+      <c r="G11" s="34">
         <f>IF(E11=0,0,F11/E11)</f>
         <v/>
       </c>
-      <c r="H11" s="32">
+      <c r="H11" s="34">
         <f>Supuestos!$C$13</f>
         <v/>
       </c>
-      <c r="I11" s="30">
+      <c r="I11" s="33">
         <f>F11*(1-H11)</f>
         <v/>
       </c>
-      <c r="J11" s="23">
+      <c r="J11" s="25">
         <f>I11*C11</f>
         <v/>
       </c>
-      <c r="K11" s="23">
+      <c r="K11" s="25">
         <f>J11*12</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="33" t="inlineStr">
+      <c r="A12" s="35" t="inlineStr">
         <is>
           <t>Argentina</t>
         </is>
       </c>
-      <c r="B12" s="33" t="inlineStr">
+      <c r="B12" s="35" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="C12" s="34">
+      <c r="C12" s="36">
         <f>Supuestos!$B$19</f>
         <v/>
       </c>
-      <c r="D12" s="35">
+      <c r="D12" s="37">
         <f>Supuestos!$B$5/C12</f>
         <v/>
       </c>
-      <c r="E12" s="35">
+      <c r="E12" s="37">
         <f>Supuestos!$E$13</f>
         <v/>
       </c>
-      <c r="F12" s="35">
+      <c r="F12" s="37">
         <f>E12-D12</f>
         <v/>
       </c>
-      <c r="G12" s="36">
+      <c r="G12" s="38">
         <f>IF(E12=0,0,F12/E12)</f>
         <v/>
       </c>
-      <c r="H12" s="36">
+      <c r="H12" s="38">
         <f>Supuestos!$C$13</f>
         <v/>
       </c>
-      <c r="I12" s="35">
+      <c r="I12" s="37">
         <f>F12*(1-H12)</f>
         <v/>
       </c>
-      <c r="J12" s="37">
+      <c r="J12" s="39">
         <f>I12*C12</f>
         <v/>
       </c>
-      <c r="K12" s="37">
+      <c r="K12" s="39">
         <f>J12*12</f>
         <v/>
       </c>
@@ -2042,39 +2312,39 @@
           <t>Alto</t>
         </is>
       </c>
-      <c r="C13" s="24">
+      <c r="C13" s="26">
         <f>Supuestos!$B$20</f>
         <v/>
       </c>
-      <c r="D13" s="30">
+      <c r="D13" s="33">
         <f>Supuestos!$B$5/C13</f>
         <v/>
       </c>
-      <c r="E13" s="30">
+      <c r="E13" s="33">
         <f>Supuestos!$E$13</f>
         <v/>
       </c>
-      <c r="F13" s="30">
+      <c r="F13" s="33">
         <f>E13-D13</f>
         <v/>
       </c>
-      <c r="G13" s="32">
+      <c r="G13" s="34">
         <f>IF(E13=0,0,F13/E13)</f>
         <v/>
       </c>
-      <c r="H13" s="32">
+      <c r="H13" s="34">
         <f>Supuestos!$C$13</f>
         <v/>
       </c>
-      <c r="I13" s="30">
+      <c r="I13" s="33">
         <f>F13*(1-H13)</f>
         <v/>
       </c>
-      <c r="J13" s="23">
+      <c r="J13" s="25">
         <f>I13*C13</f>
         <v/>
       </c>
-      <c r="K13" s="23">
+      <c r="K13" s="25">
         <f>J13*12</f>
         <v/>
       </c>
@@ -2090,87 +2360,87 @@
           <t>Bajo</t>
         </is>
       </c>
-      <c r="C14" s="24">
+      <c r="C14" s="26">
         <f>Supuestos!$B$18</f>
         <v/>
       </c>
-      <c r="D14" s="30">
+      <c r="D14" s="33">
         <f>Supuestos!$B$5/C14</f>
         <v/>
       </c>
-      <c r="E14" s="30">
+      <c r="E14" s="33">
         <f>Supuestos!$E$14</f>
         <v/>
       </c>
-      <c r="F14" s="30">
+      <c r="F14" s="33">
         <f>E14-D14</f>
         <v/>
       </c>
-      <c r="G14" s="32">
+      <c r="G14" s="34">
         <f>IF(E14=0,0,F14/E14)</f>
         <v/>
       </c>
-      <c r="H14" s="32">
+      <c r="H14" s="34">
         <f>Supuestos!$C$14</f>
         <v/>
       </c>
-      <c r="I14" s="30">
+      <c r="I14" s="33">
         <f>F14*(1-H14)</f>
         <v/>
       </c>
-      <c r="J14" s="23">
+      <c r="J14" s="25">
         <f>I14*C14</f>
         <v/>
       </c>
-      <c r="K14" s="23">
+      <c r="K14" s="25">
         <f>J14*12</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="33" t="inlineStr">
+      <c r="A15" s="35" t="inlineStr">
         <is>
           <t>Colombia</t>
         </is>
       </c>
-      <c r="B15" s="33" t="inlineStr">
+      <c r="B15" s="35" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="C15" s="34">
+      <c r="C15" s="36">
         <f>Supuestos!$B$19</f>
         <v/>
       </c>
-      <c r="D15" s="35">
+      <c r="D15" s="37">
         <f>Supuestos!$B$5/C15</f>
         <v/>
       </c>
-      <c r="E15" s="35">
+      <c r="E15" s="37">
         <f>Supuestos!$E$14</f>
         <v/>
       </c>
-      <c r="F15" s="35">
+      <c r="F15" s="37">
         <f>E15-D15</f>
         <v/>
       </c>
-      <c r="G15" s="36">
+      <c r="G15" s="38">
         <f>IF(E15=0,0,F15/E15)</f>
         <v/>
       </c>
-      <c r="H15" s="36">
+      <c r="H15" s="38">
         <f>Supuestos!$C$14</f>
         <v/>
       </c>
-      <c r="I15" s="35">
+      <c r="I15" s="37">
         <f>F15*(1-H15)</f>
         <v/>
       </c>
-      <c r="J15" s="37">
+      <c r="J15" s="39">
         <f>I15*C15</f>
         <v/>
       </c>
-      <c r="K15" s="37">
+      <c r="K15" s="39">
         <f>J15*12</f>
         <v/>
       </c>
@@ -2186,39 +2456,39 @@
           <t>Alto</t>
         </is>
       </c>
-      <c r="C16" s="24">
+      <c r="C16" s="26">
         <f>Supuestos!$B$20</f>
         <v/>
       </c>
-      <c r="D16" s="30">
+      <c r="D16" s="33">
         <f>Supuestos!$B$5/C16</f>
         <v/>
       </c>
-      <c r="E16" s="30">
+      <c r="E16" s="33">
         <f>Supuestos!$E$14</f>
         <v/>
       </c>
-      <c r="F16" s="30">
+      <c r="F16" s="33">
         <f>E16-D16</f>
         <v/>
       </c>
-      <c r="G16" s="32">
+      <c r="G16" s="34">
         <f>IF(E16=0,0,F16/E16)</f>
         <v/>
       </c>
-      <c r="H16" s="32">
+      <c r="H16" s="34">
         <f>Supuestos!$C$14</f>
         <v/>
       </c>
-      <c r="I16" s="30">
+      <c r="I16" s="33">
         <f>F16*(1-H16)</f>
         <v/>
       </c>
-      <c r="J16" s="23">
+      <c r="J16" s="25">
         <f>I16*C16</f>
         <v/>
       </c>
-      <c r="K16" s="23">
+      <c r="K16" s="25">
         <f>J16*12</f>
         <v/>
       </c>
@@ -2234,87 +2504,87 @@
           <t>Bajo</t>
         </is>
       </c>
-      <c r="C17" s="24">
+      <c r="C17" s="26">
         <f>Supuestos!$B$18</f>
         <v/>
       </c>
-      <c r="D17" s="30">
+      <c r="D17" s="33">
         <f>Supuestos!$B$5/C17</f>
         <v/>
       </c>
-      <c r="E17" s="30">
+      <c r="E17" s="33">
         <f>Supuestos!$E$15</f>
         <v/>
       </c>
-      <c r="F17" s="30">
+      <c r="F17" s="33">
         <f>E17-D17</f>
         <v/>
       </c>
-      <c r="G17" s="32">
+      <c r="G17" s="34">
         <f>IF(E17=0,0,F17/E17)</f>
         <v/>
       </c>
-      <c r="H17" s="32">
+      <c r="H17" s="34">
         <f>Supuestos!$C$15</f>
         <v/>
       </c>
-      <c r="I17" s="30">
+      <c r="I17" s="33">
         <f>F17*(1-H17)</f>
         <v/>
       </c>
-      <c r="J17" s="23">
+      <c r="J17" s="25">
         <f>I17*C17</f>
         <v/>
       </c>
-      <c r="K17" s="23">
+      <c r="K17" s="25">
         <f>J17*12</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="33" t="inlineStr">
+      <c r="A18" s="35" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="B18" s="33" t="inlineStr">
+      <c r="B18" s="35" t="inlineStr">
         <is>
           <t>Medio</t>
         </is>
       </c>
-      <c r="C18" s="34">
+      <c r="C18" s="36">
         <f>Supuestos!$B$19</f>
         <v/>
       </c>
-      <c r="D18" s="35">
+      <c r="D18" s="37">
         <f>Supuestos!$B$5/C18</f>
         <v/>
       </c>
-      <c r="E18" s="35">
+      <c r="E18" s="37">
         <f>Supuestos!$E$15</f>
         <v/>
       </c>
-      <c r="F18" s="35">
+      <c r="F18" s="37">
         <f>E18-D18</f>
         <v/>
       </c>
-      <c r="G18" s="36">
+      <c r="G18" s="38">
         <f>IF(E18=0,0,F18/E18)</f>
         <v/>
       </c>
-      <c r="H18" s="36">
+      <c r="H18" s="38">
         <f>Supuestos!$C$15</f>
         <v/>
       </c>
-      <c r="I18" s="35">
+      <c r="I18" s="37">
         <f>F18*(1-H18)</f>
         <v/>
       </c>
-      <c r="J18" s="37">
+      <c r="J18" s="39">
         <f>I18*C18</f>
         <v/>
       </c>
-      <c r="K18" s="37">
+      <c r="K18" s="39">
         <f>J18*12</f>
         <v/>
       </c>
@@ -2330,39 +2600,39 @@
           <t>Alto</t>
         </is>
       </c>
-      <c r="C19" s="24">
+      <c r="C19" s="26">
         <f>Supuestos!$B$20</f>
         <v/>
       </c>
-      <c r="D19" s="30">
+      <c r="D19" s="33">
         <f>Supuestos!$B$5/C19</f>
         <v/>
       </c>
-      <c r="E19" s="30">
+      <c r="E19" s="33">
         <f>Supuestos!$E$15</f>
         <v/>
       </c>
-      <c r="F19" s="30">
+      <c r="F19" s="33">
         <f>E19-D19</f>
         <v/>
       </c>
-      <c r="G19" s="32">
+      <c r="G19" s="34">
         <f>IF(E19=0,0,F19/E19)</f>
         <v/>
       </c>
-      <c r="H19" s="32">
+      <c r="H19" s="34">
         <f>Supuestos!$C$15</f>
         <v/>
       </c>
-      <c r="I19" s="30">
+      <c r="I19" s="33">
         <f>F19*(1-H19)</f>
         <v/>
       </c>
-      <c r="J19" s="23">
+      <c r="J19" s="25">
         <f>I19*C19</f>
         <v/>
       </c>
-      <c r="K19" s="23">
+      <c r="K19" s="25">
         <f>J19*12</f>
         <v/>
       </c>
@@ -2457,19 +2727,19 @@
           <t>Chile</t>
         </is>
       </c>
-      <c r="B5" s="23">
+      <c r="B5" s="25">
         <f>'Modelo por Estudio'!K5</f>
         <v/>
       </c>
-      <c r="C5" s="23">
+      <c r="C5" s="25">
         <f>'Modelo por Estudio'!K6</f>
         <v/>
       </c>
-      <c r="D5" s="23">
+      <c r="D5" s="25">
         <f>'Modelo por Estudio'!K7</f>
         <v/>
       </c>
-      <c r="E5" s="24">
+      <c r="E5" s="26">
         <f>Supuestos!$B$5/Supuestos!$E$11</f>
         <v/>
       </c>
@@ -2484,19 +2754,19 @@
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="B6" s="23">
+      <c r="B6" s="25">
         <f>'Modelo por Estudio'!K8</f>
         <v/>
       </c>
-      <c r="C6" s="23">
+      <c r="C6" s="25">
         <f>'Modelo por Estudio'!K9</f>
         <v/>
       </c>
-      <c r="D6" s="23">
+      <c r="D6" s="25">
         <f>'Modelo por Estudio'!K10</f>
         <v/>
       </c>
-      <c r="E6" s="24">
+      <c r="E6" s="26">
         <f>Supuestos!$B$5/Supuestos!$E$12</f>
         <v/>
       </c>
@@ -2511,19 +2781,19 @@
           <t>Argentina</t>
         </is>
       </c>
-      <c r="B7" s="23">
+      <c r="B7" s="25">
         <f>'Modelo por Estudio'!K11</f>
         <v/>
       </c>
-      <c r="C7" s="23">
+      <c r="C7" s="25">
         <f>'Modelo por Estudio'!K12</f>
         <v/>
       </c>
-      <c r="D7" s="23">
+      <c r="D7" s="25">
         <f>'Modelo por Estudio'!K13</f>
         <v/>
       </c>
-      <c r="E7" s="24">
+      <c r="E7" s="26">
         <f>Supuestos!$B$5/Supuestos!$E$13</f>
         <v/>
       </c>
@@ -2538,19 +2808,19 @@
           <t>Colombia</t>
         </is>
       </c>
-      <c r="B8" s="23">
+      <c r="B8" s="25">
         <f>'Modelo por Estudio'!K14</f>
         <v/>
       </c>
-      <c r="C8" s="23">
+      <c r="C8" s="25">
         <f>'Modelo por Estudio'!K15</f>
         <v/>
       </c>
-      <c r="D8" s="23">
+      <c r="D8" s="25">
         <f>'Modelo por Estudio'!K16</f>
         <v/>
       </c>
-      <c r="E8" s="24">
+      <c r="E8" s="26">
         <f>Supuestos!$B$5/Supuestos!$E$14</f>
         <v/>
       </c>
@@ -2565,19 +2835,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="B9" s="23">
+      <c r="B9" s="25">
         <f>'Modelo por Estudio'!K17</f>
         <v/>
       </c>
-      <c r="C9" s="23">
+      <c r="C9" s="25">
         <f>'Modelo por Estudio'!K18</f>
         <v/>
       </c>
-      <c r="D9" s="23">
+      <c r="D9" s="25">
         <f>'Modelo por Estudio'!K19</f>
         <v/>
       </c>
-      <c r="E9" s="24">
+      <c r="E9" s="26">
         <f>Supuestos!$B$5/Supuestos!$E$15</f>
         <v/>
       </c>
@@ -2587,25 +2857,25 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="27" t="inlineStr">
         <is>
           <t>Promedio</t>
         </is>
       </c>
-      <c r="B10" s="28">
+      <c r="B10" s="30">
         <f>AVERAGE(B5:B9)</f>
         <v/>
       </c>
-      <c r="C10" s="28">
+      <c r="C10" s="30">
         <f>AVERAGE(C5:C9)</f>
         <v/>
       </c>
-      <c r="D10" s="28">
+      <c r="D10" s="30">
         <f>AVERAGE(D5:D9)</f>
         <v/>
       </c>
-      <c r="E10" s="38" t="n"/>
-      <c r="F10" s="38" t="n"/>
+      <c r="E10" s="40" t="n"/>
+      <c r="F10" s="40" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2696,11 +2966,11 @@
           <t>Chile</t>
         </is>
       </c>
-      <c r="B5" s="23">
+      <c r="B5" s="25">
         <f>Supuestos!$D$11</f>
         <v/>
       </c>
-      <c r="C5" s="30">
+      <c r="C5" s="33">
         <f>Supuestos!$E$11</f>
         <v/>
       </c>
@@ -2708,15 +2978,15 @@
         <f>Supuestos!$F$11</f>
         <v/>
       </c>
-      <c r="E5" s="24">
+      <c r="E5" s="26">
         <f>Supuestos!$B$5/Supuestos!$E$11</f>
         <v/>
       </c>
-      <c r="F5" s="30">
+      <c r="F5" s="33">
         <f>'Modelo por Estudio'!I6</f>
         <v/>
       </c>
-      <c r="G5" s="23">
+      <c r="G5" s="25">
         <f>'Modelo por Estudio'!K6</f>
         <v/>
       </c>
@@ -2727,11 +2997,11 @@
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="B6" s="23">
+      <c r="B6" s="25">
         <f>Supuestos!$D$12</f>
         <v/>
       </c>
-      <c r="C6" s="30">
+      <c r="C6" s="33">
         <f>Supuestos!$E$12</f>
         <v/>
       </c>
@@ -2739,46 +3009,46 @@
         <f>Supuestos!$F$12</f>
         <v/>
       </c>
-      <c r="E6" s="24">
+      <c r="E6" s="26">
         <f>Supuestos!$B$5/Supuestos!$E$12</f>
         <v/>
       </c>
-      <c r="F6" s="30">
+      <c r="F6" s="33">
         <f>'Modelo por Estudio'!I9</f>
         <v/>
       </c>
-      <c r="G6" s="23">
+      <c r="G6" s="25">
         <f>'Modelo por Estudio'!K9</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="39" t="inlineStr">
+      <c r="A7" s="41" t="inlineStr">
         <is>
           <t>Argentina</t>
         </is>
       </c>
-      <c r="B7" s="40">
+      <c r="B7" s="42">
         <f>Supuestos!$D$13</f>
         <v/>
       </c>
-      <c r="C7" s="41">
+      <c r="C7" s="43">
         <f>Supuestos!$E$13</f>
         <v/>
       </c>
-      <c r="D7" s="42">
+      <c r="D7" s="44">
         <f>Supuestos!$F$13</f>
         <v/>
       </c>
-      <c r="E7" s="43">
+      <c r="E7" s="45">
         <f>Supuestos!$B$5/Supuestos!$E$13</f>
         <v/>
       </c>
-      <c r="F7" s="41">
+      <c r="F7" s="43">
         <f>'Modelo por Estudio'!I12</f>
         <v/>
       </c>
-      <c r="G7" s="40">
+      <c r="G7" s="42">
         <f>'Modelo por Estudio'!K12</f>
         <v/>
       </c>
@@ -2789,11 +3059,11 @@
           <t>Colombia</t>
         </is>
       </c>
-      <c r="B8" s="23">
+      <c r="B8" s="25">
         <f>Supuestos!$D$14</f>
         <v/>
       </c>
-      <c r="C8" s="30">
+      <c r="C8" s="33">
         <f>Supuestos!$E$14</f>
         <v/>
       </c>
@@ -2801,15 +3071,15 @@
         <f>Supuestos!$F$14</f>
         <v/>
       </c>
-      <c r="E8" s="24">
+      <c r="E8" s="26">
         <f>Supuestos!$B$5/Supuestos!$E$14</f>
         <v/>
       </c>
-      <c r="F8" s="30">
+      <c r="F8" s="33">
         <f>'Modelo por Estudio'!I15</f>
         <v/>
       </c>
-      <c r="G8" s="23">
+      <c r="G8" s="25">
         <f>'Modelo por Estudio'!K15</f>
         <v/>
       </c>
@@ -2820,11 +3090,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="B9" s="23">
+      <c r="B9" s="25">
         <f>Supuestos!$D$15</f>
         <v/>
       </c>
-      <c r="C9" s="30">
+      <c r="C9" s="33">
         <f>Supuestos!$E$15</f>
         <v/>
       </c>
@@ -2832,15 +3102,15 @@
         <f>Supuestos!$F$15</f>
         <v/>
       </c>
-      <c r="E9" s="24">
+      <c r="E9" s="26">
         <f>Supuestos!$B$5/Supuestos!$E$15</f>
         <v/>
       </c>
-      <c r="F9" s="30">
+      <c r="F9" s="33">
         <f>'Modelo por Estudio'!I18</f>
         <v/>
       </c>
-      <c r="G9" s="23">
+      <c r="G9" s="25">
         <f>'Modelo por Estudio'!K18</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Calculadora: costos fijos del documento, fiscalidad corregida y resultados agrupados
- Costos Rumotech fijos según la propuesta adjunta (SaaS 100/mes por modalidad y
  sede; EBOX 833/mes por resonador + 175/mes por modalidad adicional). Ya no son
  editables: la palanca simulable es el precio de venta.
- IIBB sobre la factura completa (precio de venta + IVA); ganancias sobre el
  margen (precio de venta - costo del servicio); IVA trasladado, neutro.
- Títulos corregidos (Ingreso bruto, no neto) y resultados agrupados en precios,
  ingresos, costos, impuestos y resultado, con pie de explicación por dato.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modelo.xlsx
+++ b/modelo.xlsx
@@ -241,10 +241,10 @@
     <xf numFmtId="3" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -438,74 +438,104 @@
         <t>RM: con SaaS+Cryo = costo fijo por sede; con EBOX = (costo anual EBOX ÷ 12) × resonadores de la sede.</t>
       </text>
     </comment>
-    <comment ref="A22" authorId="0" shapeId="0">
+    <comment ref="E15" authorId="0" shapeId="0">
       <text>
-        <t>Modalidades distintas por sede. Cada una paga el costo fijo (salvo RM con EBOX).</t>
+        <t>Modalidad adicional (según la propuesta Rumotech): con SaaS Full + Cryogenics = USD 1.200/año = USD 100/mes; con EBOX Full = USD 2.100/año = USD 175/mes.</t>
+      </text>
+    </comment>
+    <comment ref="E16" authorId="0" shapeId="0">
+      <text>
+        <t>Modalidad adicional (según la propuesta Rumotech): con SaaS Full + Cryogenics = USD 1.200/año = USD 100/mes; con EBOX Full = USD 2.100/año = USD 175/mes.</t>
+      </text>
+    </comment>
+    <comment ref="E17" authorId="0" shapeId="0">
+      <text>
+        <t>Modalidad adicional (según la propuesta Rumotech): con SaaS Full + Cryogenics = USD 1.200/año = USD 100/mes; con EBOX Full = USD 2.100/año = USD 175/mes.</t>
+      </text>
+    </comment>
+    <comment ref="E18" authorId="0" shapeId="0">
+      <text>
+        <t>Modalidad adicional (según la propuesta Rumotech): con SaaS Full + Cryogenics = USD 1.200/año = USD 100/mes; con EBOX Full = USD 2.100/año = USD 175/mes.</t>
       </text>
     </comment>
     <comment ref="A23" authorId="0" shapeId="0">
       <text>
-        <t>Por equipos = Σ equipos × estudios. Por pacientes = pacientes × coeficiente.</t>
+        <t>Lo que le cobramos al centro por cada estudio, sin IVA. Es la palanca que se simula (editable en Supuestos, por país).</t>
       </text>
     </comment>
     <comment ref="A24" authorId="0" shapeId="0">
       <text>
-        <t>Prestaciones por sede × número de sedes.</t>
+        <t>Precio de venta × IVA del país. Se le suma al cliente en la factura y se traslada al fisco.</t>
       </text>
     </comment>
     <comment ref="A25" authorId="0" shapeId="0">
       <text>
-        <t>Suma de costos por modalidad y sede. RM con EBOX = (costo anual÷12) × resonadores.</t>
-      </text>
-    </comment>
-    <comment ref="A26" authorId="0" shapeId="0">
-      <text>
-        <t>Costo total ÷ prestaciones. Baja con la densidad de equipos/sedes.</t>
+        <t>Precio de venta + IVA. Es lo que el cliente paga por cada estudio.</t>
       </text>
     </comment>
     <comment ref="A27" authorId="0" shapeId="0">
       <text>
-        <t>Precio de venta al centro, sin IVA. Se toma de Supuestos según el país.</t>
+        <t>Por equipos = Σ equipos × estudios/equipo. Por pacientes = pacientes × coeficiente.</t>
       </text>
     </comment>
     <comment ref="A28" authorId="0" shapeId="0">
       <text>
-        <t>Precio × (1 + IVA). El IVA es pass-through: neutro para la renta.</t>
+        <t>Prestaciones por sede × número de sedes.</t>
       </text>
     </comment>
     <comment ref="A29" authorId="0" shapeId="0">
       <text>
-        <t>Volumen total × precio neto de IVA.</t>
+        <t>Volumen total × precio de venta. Es facturación antes de costos e impuestos: NO es ganancia.</t>
       </text>
     </comment>
     <comment ref="A30" authorId="0" shapeId="0">
       <text>
-        <t>Impuesto provincial argentino sobre el ingreso bruto. Reduce el margen. 0 en los demás países.</t>
-      </text>
-    </comment>
-    <comment ref="A31" authorId="0" shapeId="0">
-      <text>
-        <t>Ingreso − costo Rumotech − IIBB.</t>
+        <t>Ingreso bruto + IVA. Es el total que se le cobra al cliente y la BASE del IIBB.</t>
       </text>
     </comment>
     <comment ref="A32" authorId="0" shapeId="0">
       <text>
-        <t>Alícuota del país sobre el margen operativo positivo.</t>
+        <t>Fijo según la propuesta: SaaS Full+Cryogenics USD 100/mes por modalidad y sede; EBOX Full USD 833/mes por resonador + USD 175/mes por modalidad adicional. No editable.</t>
       </text>
     </comment>
     <comment ref="A33" authorId="0" shapeId="0">
       <text>
-        <t>Costo único por resonador: SaaS+Cryo 150, EBOX 500. No es recurrente; no entra en la renta anual.</t>
+        <t>Costo Rumotech ÷ prestaciones. Baja al sumar equipos o sedes: la densidad diluye el costo fijo.</t>
       </text>
     </comment>
     <comment ref="A34" authorId="0" shapeId="0">
       <text>
-        <t>Margen operativo menos impuesto a la renta.</t>
+        <t>Pago único por resonador: SaaS+Cryogenics USD 150, EBOX USD 500. No entra en la ganancia recurrente.</t>
       </text>
     </comment>
-    <comment ref="A35" authorId="0" shapeId="0">
+    <comment ref="A36" authorId="0" shapeId="0">
       <text>
-        <t>Renta pasiva anual que retiene NexoLibre.</t>
+        <t>Ingreso bruto × IVA. Lo paga el cliente y se traslada al fisco: NO afecta nuestra ganancia.</t>
+      </text>
+    </comment>
+    <comment ref="A37" authorId="0" shapeId="0">
+      <text>
+        <t>Factura completa (precio de venta + IVA) × IIBB%. Se aplica sobre la factura CON IVA incluido. Sí es costo nuestro. 0 fuera de Argentina.</t>
+      </text>
+    </comment>
+    <comment ref="A38" authorId="0" shapeId="0">
+      <text>
+        <t>Margen bruto × alícuota del país. Se calcula sobre el margen: precio de venta − costo del servicio.</t>
+      </text>
+    </comment>
+    <comment ref="A40" authorId="0" shapeId="0">
+      <text>
+        <t>Ingreso bruto − costo Rumotech. Antes de impuestos.</t>
+      </text>
+    </comment>
+    <comment ref="A41" authorId="0" shapeId="0">
+      <text>
+        <t>Margen bruto − IIBB − impuesto a las ganancias.</t>
+      </text>
+    </comment>
+    <comment ref="A42" authorId="0" shapeId="0">
+      <text>
+        <t>Ganancia neta mensual × 12. Es la renta pasiva que retiene NexoLibre por este cliente.</t>
       </text>
     </comment>
   </commentList>
@@ -1293,7 +1323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1480,7 +1510,7 @@
         <v/>
       </c>
       <c r="E15" s="25">
-        <f>IF(B15&gt;0,Supuestos!$B$5,0)</f>
+        <f>IF(B15&gt;0,IF($B$7="EBOX Full",2100/12,Supuestos!$B$5),0)</f>
         <v/>
       </c>
       <c r="F15" s="26">
@@ -1505,7 +1535,7 @@
         <v/>
       </c>
       <c r="E16" s="25">
-        <f>IF(B16&gt;0,Supuestos!$B$5,0)</f>
+        <f>IF(B16&gt;0,IF($B$7="EBOX Full",2100/12,Supuestos!$B$5),0)</f>
         <v/>
       </c>
       <c r="F16" s="26">
@@ -1530,7 +1560,7 @@
         <v/>
       </c>
       <c r="E17" s="25">
-        <f>IF(B17&gt;0,Supuestos!$B$5,0)</f>
+        <f>IF(B17&gt;0,IF($B$7="EBOX Full",2100/12,Supuestos!$B$5),0)</f>
         <v/>
       </c>
       <c r="F17" s="26">
@@ -1555,7 +1585,7 @@
         <v/>
       </c>
       <c r="E18" s="25">
-        <f>IF(B18&gt;0,Supuestos!$B$5,0)</f>
+        <f>IF(B18&gt;0,IF($B$7="EBOX Full",2100/12,Supuestos!$B$5),0)</f>
         <v/>
       </c>
       <c r="F18" s="26">
@@ -1592,25 +1622,20 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Modalidades activas por sede</t>
-        </is>
-      </c>
-      <c r="E22" s="26">
-        <f>D19</f>
-        <v/>
-      </c>
-      <c r="F22" s="7" t="n"/>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>1 · PRECIOS DE VENTA</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Prestaciones (estudios) por sede</t>
-        </is>
-      </c>
-      <c r="E23" s="26">
-        <f>IF($B$9="Por pacientes",$B$10*$B$11,F19)</f>
+          <t>Precio de venta por prestación (sin IVA)</t>
+        </is>
+      </c>
+      <c r="E23" s="32">
+        <f>INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))</f>
         <v/>
       </c>
       <c r="F23" s="7" t="n"/>
@@ -1618,11 +1643,11 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Volumen total de prestaciones / mes</t>
-        </is>
-      </c>
-      <c r="E24" s="26">
-        <f>(IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6</f>
+          <t>IVA por prestación</t>
+        </is>
+      </c>
+      <c r="E24" s="32">
+        <f>E23*INDEX(Supuestos!$B$11:$B$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))</f>
         <v/>
       </c>
       <c r="F24" s="7" t="n"/>
@@ -1630,35 +1655,30 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Costo Rumotech mensual — total (USD)</t>
-        </is>
-      </c>
-      <c r="E25" s="25">
-        <f>E19*$B$6</f>
+          <t>Precio facturado por prestación (c/IVA)</t>
+        </is>
+      </c>
+      <c r="E25" s="32">
+        <f>E23+E24</f>
         <v/>
       </c>
       <c r="F25" s="7" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Costo Rumotech EFECTIVO por prestación (USD)</t>
-        </is>
-      </c>
-      <c r="E26" s="32">
-        <f>IF(((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)=0,0,(E19*$B$6)/((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6))</f>
-        <v/>
-      </c>
-      <c r="F26" s="7" t="n"/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2 · INGRESOS</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Precio por prestación — neto de IVA (USD)</t>
-        </is>
-      </c>
-      <c r="E27" s="33">
-        <f>INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))</f>
+          <t>Prestaciones por sede / mes</t>
+        </is>
+      </c>
+      <c r="E27" s="26">
+        <f>IF($B$9="Por pacientes",$B$10*$B$11,F19)</f>
         <v/>
       </c>
       <c r="F27" s="7" t="n"/>
@@ -1666,11 +1686,11 @@
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Precio final al cliente c/ IVA (USD)</t>
-        </is>
-      </c>
-      <c r="E28" s="33">
-        <f>INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))*(1+INDEX(Supuestos!$B$11:$B$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))</f>
+          <t>Volumen total de prestaciones / mes</t>
+        </is>
+      </c>
+      <c r="E28" s="26">
+        <f>E27*$B$6</f>
         <v/>
       </c>
       <c r="F28" s="7" t="n"/>
@@ -1678,11 +1698,11 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Ingreso mensual — total (USD)</t>
+          <t>Ingreso BRUTO / mes (sin IVA)</t>
         </is>
       </c>
       <c r="E29" s="25">
-        <f>((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))</f>
+        <f>E28*E23</f>
         <v/>
       </c>
       <c r="F29" s="7" t="n"/>
@@ -1690,35 +1710,30 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Ingresos Brutos (IIBB) mensual (USD)</t>
+          <t>Facturación total / mes (c/IVA)</t>
         </is>
       </c>
       <c r="E30" s="25">
-        <f>(((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))</f>
+        <f>E29*(1+INDEX(Supuestos!$B$11:$B$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))</f>
         <v/>
       </c>
       <c r="F30" s="7" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>Margen operativo mensual (USD)</t>
-        </is>
-      </c>
-      <c r="E31" s="25">
-        <f>(((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))-(E19*$B$6)-((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))</f>
-        <v/>
-      </c>
-      <c r="F31" s="7" t="n"/>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>3 · COSTOS  (fijos — según la propuesta Rumotech adjunta)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Impuesto a la renta mensual (USD)</t>
+          <t>Costo Rumotech / mes — total</t>
         </is>
       </c>
       <c r="E32" s="25">
-        <f>IF(((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))-(E19*$B$6)-((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))))&gt;0,((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))-(E19*$B$6)-((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))))*INDEX(Supuestos!$C$11:$C$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)),0)</f>
+        <f>E19*$B$6</f>
         <v/>
       </c>
       <c r="F32" s="7" t="n"/>
@@ -1726,11 +1741,11 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Hardware (pago ÚNICO, USD)</t>
-        </is>
-      </c>
-      <c r="E33" s="25">
-        <f>IF($B$7="EBOX Full",500,150)*B14*$B$6</f>
+          <t>Costo efectivo por prestación</t>
+        </is>
+      </c>
+      <c r="E33" s="33">
+        <f>IF(E28=0,0,E32/E28)</f>
         <v/>
       </c>
       <c r="F33" s="7" t="n"/>
@@ -1738,66 +1753,149 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Renta neta mensual (USD)</t>
+          <t>Hardware (pago ÚNICO)</t>
         </is>
       </c>
       <c r="E34" s="25">
-        <f>((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))-(E19*$B$6)-((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))))-IF(((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))-(E19*$B$6)-((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))))&gt;0,((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))-(E19*$B$6)-((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))))*INDEX(Supuestos!$C$11:$C$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)),0)</f>
+        <f>IF($B$7="EBOX Full",500,150)*B14*$B$6</f>
         <v/>
       </c>
       <c r="F34" s="7" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>RENTA NETA ANUAL — total cliente (USD)</t>
-        </is>
-      </c>
-      <c r="E35" s="6">
-        <f>(((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))-(E19*$B$6)-((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))))-IF(((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))-(E19*$B$6)-((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))))&gt;0,((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))-(E19*$B$6)-((((IF($B$9="Por pacientes",$B$10*$B$11,F19))*$B$6)*INDEX(Supuestos!$E$11:$E$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)))*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))))*INDEX(Supuestos!$C$11:$C$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)),0))*12</f>
-        <v/>
-      </c>
-      <c r="F35" s="7" t="n"/>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>4 · IMPUESTOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>IVA trasladado / mes</t>
+        </is>
+      </c>
+      <c r="E36" s="25">
+        <f>E29*INDEX(Supuestos!$B$11:$B$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))</f>
+        <v/>
+      </c>
+      <c r="F36" s="7" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>Ejercicios: cambiá el plan de RM (SaaS+Cryo vs EBOX), el método de volumen (equipos vs pacientes) o el país, y observá la renta.</t>
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Ingresos Brutos (IIBB) / mes</t>
+        </is>
+      </c>
+      <c r="E37" s="25">
+        <f>E30*INDEX(Supuestos!$G$11:$G$15,MATCH($B$5,Supuestos!$A$11:$A$15,0))</f>
+        <v/>
+      </c>
+      <c r="F37" s="7" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Impuesto a las ganancias / mes</t>
+        </is>
+      </c>
+      <c r="E38" s="25">
+        <f>IF(E40&gt;0,E40*INDEX(Supuestos!$C$11:$C$15,MATCH($B$5,Supuestos!$A$11:$A$15,0)),0)</f>
+        <v/>
+      </c>
+      <c r="F38" s="7" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>5 · RESULTADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Margen bruto / mes</t>
+        </is>
+      </c>
+      <c r="E40" s="25">
+        <f>E29-E32</f>
+        <v/>
+      </c>
+      <c r="F40" s="7" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>GANANCIA NETA / mes</t>
+        </is>
+      </c>
+      <c r="E41" s="6">
+        <f>E40-E37-E38</f>
+        <v/>
+      </c>
+      <c r="F41" s="7" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>GANANCIA NETA ANUAL — total cliente</t>
+        </is>
+      </c>
+      <c r="E42" s="6">
+        <f>E41*12</f>
+        <v/>
+      </c>
+      <c r="F42" s="7" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Cada etiqueta tiene un comentario (triángulo rojo) que explica el dato y su fórmula. Ejercicios: cambiá el plan de RM, el método de volumen o el país.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="31">
+  <mergeCells count="40">
     <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A22:D22"/>
     <mergeCell ref="E24:F24"/>
-    <mergeCell ref="A35:D35"/>
     <mergeCell ref="E33:F33"/>
-    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A38:D38"/>
     <mergeCell ref="A29:D29"/>
     <mergeCell ref="E23:F23"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="A26:F26"/>
     <mergeCell ref="A28:D28"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="E38:F38"/>
     <mergeCell ref="E29:F29"/>
     <mergeCell ref="A34:D34"/>
     <mergeCell ref="A30:D30"/>
     <mergeCell ref="E28:F28"/>
+    <mergeCell ref="A22:F22"/>
     <mergeCell ref="A24:D24"/>
-    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="A36:D36"/>
     <mergeCell ref="E34:F34"/>
     <mergeCell ref="E30:F30"/>
+    <mergeCell ref="A44:F44"/>
     <mergeCell ref="E27:F27"/>
+    <mergeCell ref="A31:F31"/>
     <mergeCell ref="A25:D25"/>
-    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A39:F39"/>
+    <mergeCell ref="A37:D37"/>
     <mergeCell ref="A27:D27"/>
     <mergeCell ref="E32:F32"/>
     <mergeCell ref="E25:F25"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="E37:F37"/>
     <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A42:D42"/>
     <mergeCell ref="A32:D32"/>
   </mergeCells>
   <dataValidations count="3">
@@ -1932,15 +2030,15 @@
         <f>Supuestos!$B$18</f>
         <v/>
       </c>
-      <c r="D5" s="33">
+      <c r="D5" s="32">
         <f>Supuestos!$B$5/C5</f>
         <v/>
       </c>
-      <c r="E5" s="33">
+      <c r="E5" s="32">
         <f>Supuestos!$E$11</f>
         <v/>
       </c>
-      <c r="F5" s="33">
+      <c r="F5" s="32">
         <f>E5-D5</f>
         <v/>
       </c>
@@ -1952,7 +2050,7 @@
         <f>Supuestos!$C$11</f>
         <v/>
       </c>
-      <c r="I5" s="33">
+      <c r="I5" s="32">
         <f>F5*(1-H5)</f>
         <v/>
       </c>
@@ -2028,15 +2126,15 @@
         <f>Supuestos!$B$20</f>
         <v/>
       </c>
-      <c r="D7" s="33">
+      <c r="D7" s="32">
         <f>Supuestos!$B$5/C7</f>
         <v/>
       </c>
-      <c r="E7" s="33">
+      <c r="E7" s="32">
         <f>Supuestos!$E$11</f>
         <v/>
       </c>
-      <c r="F7" s="33">
+      <c r="F7" s="32">
         <f>E7-D7</f>
         <v/>
       </c>
@@ -2048,7 +2146,7 @@
         <f>Supuestos!$C$11</f>
         <v/>
       </c>
-      <c r="I7" s="33">
+      <c r="I7" s="32">
         <f>F7*(1-H7)</f>
         <v/>
       </c>
@@ -2076,15 +2174,15 @@
         <f>Supuestos!$B$18</f>
         <v/>
       </c>
-      <c r="D8" s="33">
+      <c r="D8" s="32">
         <f>Supuestos!$B$5/C8</f>
         <v/>
       </c>
-      <c r="E8" s="33">
+      <c r="E8" s="32">
         <f>Supuestos!$E$12</f>
         <v/>
       </c>
-      <c r="F8" s="33">
+      <c r="F8" s="32">
         <f>E8-D8</f>
         <v/>
       </c>
@@ -2096,7 +2194,7 @@
         <f>Supuestos!$C$12</f>
         <v/>
       </c>
-      <c r="I8" s="33">
+      <c r="I8" s="32">
         <f>F8*(1-H8)</f>
         <v/>
       </c>
@@ -2172,15 +2270,15 @@
         <f>Supuestos!$B$20</f>
         <v/>
       </c>
-      <c r="D10" s="33">
+      <c r="D10" s="32">
         <f>Supuestos!$B$5/C10</f>
         <v/>
       </c>
-      <c r="E10" s="33">
+      <c r="E10" s="32">
         <f>Supuestos!$E$12</f>
         <v/>
       </c>
-      <c r="F10" s="33">
+      <c r="F10" s="32">
         <f>E10-D10</f>
         <v/>
       </c>
@@ -2192,7 +2290,7 @@
         <f>Supuestos!$C$12</f>
         <v/>
       </c>
-      <c r="I10" s="33">
+      <c r="I10" s="32">
         <f>F10*(1-H10)</f>
         <v/>
       </c>
@@ -2220,15 +2318,15 @@
         <f>Supuestos!$B$18</f>
         <v/>
       </c>
-      <c r="D11" s="33">
+      <c r="D11" s="32">
         <f>Supuestos!$B$5/C11</f>
         <v/>
       </c>
-      <c r="E11" s="33">
+      <c r="E11" s="32">
         <f>Supuestos!$E$13</f>
         <v/>
       </c>
-      <c r="F11" s="33">
+      <c r="F11" s="32">
         <f>E11-D11</f>
         <v/>
       </c>
@@ -2240,7 +2338,7 @@
         <f>Supuestos!$C$13</f>
         <v/>
       </c>
-      <c r="I11" s="33">
+      <c r="I11" s="32">
         <f>F11*(1-H11)</f>
         <v/>
       </c>
@@ -2316,15 +2414,15 @@
         <f>Supuestos!$B$20</f>
         <v/>
       </c>
-      <c r="D13" s="33">
+      <c r="D13" s="32">
         <f>Supuestos!$B$5/C13</f>
         <v/>
       </c>
-      <c r="E13" s="33">
+      <c r="E13" s="32">
         <f>Supuestos!$E$13</f>
         <v/>
       </c>
-      <c r="F13" s="33">
+      <c r="F13" s="32">
         <f>E13-D13</f>
         <v/>
       </c>
@@ -2336,7 +2434,7 @@
         <f>Supuestos!$C$13</f>
         <v/>
       </c>
-      <c r="I13" s="33">
+      <c r="I13" s="32">
         <f>F13*(1-H13)</f>
         <v/>
       </c>
@@ -2364,15 +2462,15 @@
         <f>Supuestos!$B$18</f>
         <v/>
       </c>
-      <c r="D14" s="33">
+      <c r="D14" s="32">
         <f>Supuestos!$B$5/C14</f>
         <v/>
       </c>
-      <c r="E14" s="33">
+      <c r="E14" s="32">
         <f>Supuestos!$E$14</f>
         <v/>
       </c>
-      <c r="F14" s="33">
+      <c r="F14" s="32">
         <f>E14-D14</f>
         <v/>
       </c>
@@ -2384,7 +2482,7 @@
         <f>Supuestos!$C$14</f>
         <v/>
       </c>
-      <c r="I14" s="33">
+      <c r="I14" s="32">
         <f>F14*(1-H14)</f>
         <v/>
       </c>
@@ -2460,15 +2558,15 @@
         <f>Supuestos!$B$20</f>
         <v/>
       </c>
-      <c r="D16" s="33">
+      <c r="D16" s="32">
         <f>Supuestos!$B$5/C16</f>
         <v/>
       </c>
-      <c r="E16" s="33">
+      <c r="E16" s="32">
         <f>Supuestos!$E$14</f>
         <v/>
       </c>
-      <c r="F16" s="33">
+      <c r="F16" s="32">
         <f>E16-D16</f>
         <v/>
       </c>
@@ -2480,7 +2578,7 @@
         <f>Supuestos!$C$14</f>
         <v/>
       </c>
-      <c r="I16" s="33">
+      <c r="I16" s="32">
         <f>F16*(1-H16)</f>
         <v/>
       </c>
@@ -2508,15 +2606,15 @@
         <f>Supuestos!$B$18</f>
         <v/>
       </c>
-      <c r="D17" s="33">
+      <c r="D17" s="32">
         <f>Supuestos!$B$5/C17</f>
         <v/>
       </c>
-      <c r="E17" s="33">
+      <c r="E17" s="32">
         <f>Supuestos!$E$15</f>
         <v/>
       </c>
-      <c r="F17" s="33">
+      <c r="F17" s="32">
         <f>E17-D17</f>
         <v/>
       </c>
@@ -2528,7 +2626,7 @@
         <f>Supuestos!$C$15</f>
         <v/>
       </c>
-      <c r="I17" s="33">
+      <c r="I17" s="32">
         <f>F17*(1-H17)</f>
         <v/>
       </c>
@@ -2604,15 +2702,15 @@
         <f>Supuestos!$B$20</f>
         <v/>
       </c>
-      <c r="D19" s="33">
+      <c r="D19" s="32">
         <f>Supuestos!$B$5/C19</f>
         <v/>
       </c>
-      <c r="E19" s="33">
+      <c r="E19" s="32">
         <f>Supuestos!$E$15</f>
         <v/>
       </c>
-      <c r="F19" s="33">
+      <c r="F19" s="32">
         <f>E19-D19</f>
         <v/>
       </c>
@@ -2624,7 +2722,7 @@
         <f>Supuestos!$C$15</f>
         <v/>
       </c>
-      <c r="I19" s="33">
+      <c r="I19" s="32">
         <f>F19*(1-H19)</f>
         <v/>
       </c>
@@ -2970,7 +3068,7 @@
         <f>Supuestos!$D$11</f>
         <v/>
       </c>
-      <c r="C5" s="33">
+      <c r="C5" s="32">
         <f>Supuestos!$E$11</f>
         <v/>
       </c>
@@ -2982,7 +3080,7 @@
         <f>Supuestos!$B$5/Supuestos!$E$11</f>
         <v/>
       </c>
-      <c r="F5" s="33">
+      <c r="F5" s="32">
         <f>'Modelo por Estudio'!I6</f>
         <v/>
       </c>
@@ -3001,7 +3099,7 @@
         <f>Supuestos!$D$12</f>
         <v/>
       </c>
-      <c r="C6" s="33">
+      <c r="C6" s="32">
         <f>Supuestos!$E$12</f>
         <v/>
       </c>
@@ -3013,7 +3111,7 @@
         <f>Supuestos!$B$5/Supuestos!$E$12</f>
         <v/>
       </c>
-      <c r="F6" s="33">
+      <c r="F6" s="32">
         <f>'Modelo por Estudio'!I9</f>
         <v/>
       </c>
@@ -3063,7 +3161,7 @@
         <f>Supuestos!$D$14</f>
         <v/>
       </c>
-      <c r="C8" s="33">
+      <c r="C8" s="32">
         <f>Supuestos!$E$14</f>
         <v/>
       </c>
@@ -3075,7 +3173,7 @@
         <f>Supuestos!$B$5/Supuestos!$E$14</f>
         <v/>
       </c>
-      <c r="F8" s="33">
+      <c r="F8" s="32">
         <f>'Modelo por Estudio'!I15</f>
         <v/>
       </c>
@@ -3094,7 +3192,7 @@
         <f>Supuestos!$D$15</f>
         <v/>
       </c>
-      <c r="C9" s="33">
+      <c r="C9" s="32">
         <f>Supuestos!$E$15</f>
         <v/>
       </c>
@@ -3106,7 +3204,7 @@
         <f>Supuestos!$B$5/Supuestos!$E$15</f>
         <v/>
       </c>
-      <c r="F9" s="33">
+      <c r="F9" s="32">
         <f>'Modelo por Estudio'!I18</f>
         <v/>
       </c>

</xml_diff>